<commit_message>
add fuzzy matching for misspelled natures
</commit_message>
<xml_diff>
--- a/nature_descriptions.xlsx
+++ b/nature_descriptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\SN3PEPF00017C28\EXCELCNV\17fe5b6f-b4ec-4887-911c-184e8c79a841\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{F87D147B-4C09-4E85-AB5F-C226DC3C317D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD2B1A7B-F774-4EB2-873F-7276D5221AA0}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="8_{F87D147B-4C09-4E85-AB5F-C226DC3C317D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A23C6CC2-9877-4F06-AD20-07FDF3E0B9E1}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{09135B44-E9BC-4796-B7D9-3AB46F4DE58F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="195">
   <si>
     <t>Code</t>
   </si>
@@ -359,6 +359,9 @@
     <t>BIKE TRAFFIC</t>
   </si>
   <si>
+    <t>Bike</t>
+  </si>
+  <si>
     <t>When officers stop someone on a bike</t>
   </si>
   <si>
@@ -597,6 +600,27 @@
   </si>
   <si>
     <t>PROP SAFEKEEP</t>
+  </si>
+  <si>
+    <t>ABANDPROP</t>
+  </si>
+  <si>
+    <t>DEAD ANIMAL</t>
+  </si>
+  <si>
+    <t>SUSPEND DRIVER</t>
+  </si>
+  <si>
+    <t>ARSON REPORT</t>
+  </si>
+  <si>
+    <t>BIKE PATROL</t>
+  </si>
+  <si>
+    <t>FRAUD IP/JO</t>
+  </si>
+  <si>
+    <t>EXPLOSION</t>
   </si>
 </sst>
 </file>
@@ -1444,7 +1468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{261BE51A-4603-4CDB-80FB-0950F5F3A62F}">
-  <dimension ref="A1:D111"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="28.42578125" customWidth="1"/>
@@ -2184,10 +2208,10 @@
         <v>106</v>
       </c>
       <c r="C59" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D59" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -2195,13 +2219,13 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C60" t="s">
         <v>102</v>
       </c>
       <c r="D60" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -2209,7 +2233,7 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C61" t="s">
         <v>102</v>
@@ -2220,13 +2244,13 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C62" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D62" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -2234,10 +2258,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C63" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2245,10 +2269,10 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C64" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -2256,10 +2280,10 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
+        <v>118</v>
+      </c>
+      <c r="C65" t="s">
         <v>117</v>
-      </c>
-      <c r="C65" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -2267,10 +2291,10 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C66" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -2278,13 +2302,13 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
+        <v>121</v>
+      </c>
+      <c r="C67" t="s">
         <v>120</v>
       </c>
-      <c r="C67" t="s">
-        <v>119</v>
-      </c>
       <c r="D67" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -2292,10 +2316,10 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C68" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -2303,10 +2327,10 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C69" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -2314,10 +2338,10 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
+        <v>126</v>
+      </c>
+      <c r="C70" t="s">
         <v>125</v>
-      </c>
-      <c r="C70" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2325,10 +2349,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C71" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -2336,10 +2360,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C72" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -2347,10 +2371,10 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C73" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -2358,10 +2382,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C74" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -2369,10 +2393,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C75" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -2380,13 +2404,13 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C76" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D76" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -2394,10 +2418,10 @@
         <v>75</v>
       </c>
       <c r="B77" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C77" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -2405,10 +2429,10 @@
         <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C78" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -2416,10 +2440,10 @@
         <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C79" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -2427,13 +2451,13 @@
         <v>78</v>
       </c>
       <c r="B80" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C80" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D80" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -2441,13 +2465,13 @@
         <v>79</v>
       </c>
       <c r="B81" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C81" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D81" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -2455,13 +2479,13 @@
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C82" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D82" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -2469,10 +2493,10 @@
         <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C83" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -2480,10 +2504,10 @@
         <v>82</v>
       </c>
       <c r="B84" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C84" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -2491,13 +2515,13 @@
         <v>83</v>
       </c>
       <c r="B85" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C85" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D85" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -2505,10 +2529,10 @@
         <v>84</v>
       </c>
       <c r="B86" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C86" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -2516,10 +2540,10 @@
         <v>85</v>
       </c>
       <c r="B87" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C87" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -2527,13 +2551,13 @@
         <v>86</v>
       </c>
       <c r="B88" t="s">
+        <v>152</v>
+      </c>
+      <c r="C88" t="s">
         <v>151</v>
       </c>
-      <c r="C88" t="s">
-        <v>150</v>
-      </c>
       <c r="D88" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -2541,13 +2565,13 @@
         <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C89" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D89" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -2555,10 +2579,10 @@
         <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C90" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -2566,13 +2590,13 @@
         <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C91" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D91" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -2580,13 +2604,13 @@
         <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C92" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D92" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -2594,10 +2618,10 @@
         <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C93" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -2605,13 +2629,13 @@
         <v>92</v>
       </c>
       <c r="B94" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C94" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D94" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -2619,10 +2643,10 @@
         <v>93</v>
       </c>
       <c r="B95" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C95" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -2630,10 +2654,10 @@
         <v>94</v>
       </c>
       <c r="B96" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C96" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -2641,10 +2665,10 @@
         <v>95</v>
       </c>
       <c r="B97" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C97" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -2652,10 +2676,10 @@
         <v>96</v>
       </c>
       <c r="B98" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C98" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -2663,10 +2687,10 @@
         <v>97</v>
       </c>
       <c r="B99" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C99" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -2674,10 +2698,10 @@
         <v>98</v>
       </c>
       <c r="B100" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C100" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -2685,10 +2709,10 @@
         <v>99</v>
       </c>
       <c r="B101" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C101" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -2696,10 +2720,10 @@
         <v>100</v>
       </c>
       <c r="B102" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C102" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -2707,10 +2731,10 @@
         <v>101</v>
       </c>
       <c r="B103" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C103" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -2718,13 +2742,13 @@
         <v>102</v>
       </c>
       <c r="B104" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D104" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -2732,13 +2756,13 @@
         <v>103</v>
       </c>
       <c r="B105" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C105" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D105" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -2746,13 +2770,13 @@
         <v>104</v>
       </c>
       <c r="B106" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C106" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D106" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -2760,10 +2784,10 @@
         <v>105</v>
       </c>
       <c r="B107" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C107" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -2771,10 +2795,10 @@
         <v>106</v>
       </c>
       <c r="B108" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C108" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -2782,7 +2806,7 @@
         <v>107</v>
       </c>
       <c r="B109" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C109" t="s">
         <v>71</v>
@@ -2793,7 +2817,7 @@
         <v>108</v>
       </c>
       <c r="B110" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C110" t="s">
         <v>74</v>
@@ -2804,10 +2828,87 @@
         <v>109</v>
       </c>
       <c r="B111" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C111" t="s">
-        <v>132</v>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
+      <c r="A112">
+        <v>110</v>
+      </c>
+      <c r="B112" t="s">
+        <v>188</v>
+      </c>
+      <c r="C112" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113">
+        <v>111</v>
+      </c>
+      <c r="B113" t="s">
+        <v>189</v>
+      </c>
+      <c r="C113" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114">
+        <v>112</v>
+      </c>
+      <c r="B114" t="s">
+        <v>190</v>
+      </c>
+      <c r="C114" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115">
+        <v>113</v>
+      </c>
+      <c r="B115" t="s">
+        <v>191</v>
+      </c>
+      <c r="C115" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116">
+        <v>114</v>
+      </c>
+      <c r="B116" t="s">
+        <v>192</v>
+      </c>
+      <c r="C116" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117">
+        <v>115</v>
+      </c>
+      <c r="B117" t="s">
+        <v>193</v>
+      </c>
+      <c r="C117" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3">
+      <c r="A118">
+        <v>116</v>
+      </c>
+      <c r="B118" t="s">
+        <v>194</v>
+      </c>
+      <c r="C118" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>